<commit_message>
Fix Framework section Names (YAML + Excel + Script)
</commit_message>
<xml_diff>
--- a/tools/excel/anssi/rec-secu-sys-ctrl-acces-phys-videoprot/anssi_rec-secu-sys-ctrl-acces-phys-videoprot_v2.2.xlsx
+++ b/tools/excel/anssi/rec-secu-sys-ctrl-acces-phys-videoprot/anssi_rec-secu-sys-ctrl-acces-phys-videoprot_v2.2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\tarkadia\projects\intuitem\ciso-assistant-community\tools\excel\anssi\rec-secu-sys-ctrl-acces-phys-videoprot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51BE9702-B38E-4C85-BC5B-45003DABF276}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E0AF98F-EBAB-4246-A1FA-3AF806A060D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2304" yWindow="636" windowWidth="19716" windowHeight="12324" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1485" yWindow="-15870" windowWidth="25440" windowHeight="15990" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="library_meta" sheetId="1" r:id="rId1"/>
@@ -1557,9 +1557,6 @@
     <t>Identifier les zones avec leurs niveaux de protection attendus</t>
   </si>
   <si>
-    <t>Niveaudesûretédeséquipementsetdesinstallationsdecontrôled'accès physique.</t>
-  </si>
-  <si>
     <t>Identifier les niveaux de sûreté adaptés aux menaces des sites</t>
   </si>
   <si>
@@ -1605,9 +1602,6 @@
     <t>Protéger les liaisons filaires</t>
   </si>
   <si>
-    <t>Connexionsentreles têtes de lecture et l'UTL</t>
-  </si>
-  <si>
     <t>Privilégier des connexions point-à-point entre les têtes de lecture et l'UTL</t>
   </si>
   <si>
@@ -1623,12 +1617,6 @@
     <t>Activer un deuxième chiffrement dans le cas d'une connectivité sans-fil</t>
   </si>
   <si>
-    <t>Réseausupport</t>
-  </si>
-  <si>
-    <t>Segmentationauseinduréseausupport</t>
-  </si>
-  <si>
     <t>Cloisonner logiquement les dispositifs au sein du réseau support</t>
   </si>
   <si>
@@ -1647,33 +1635,21 @@
     <t>Contrôler les accès aux ports réseau par vérification des adresses MAC</t>
   </si>
   <si>
-    <t>Mutualisationdesdispositifsdecontrôled'accèsphysiquesurunmêmeréseau support</t>
-  </si>
-  <si>
     <t>Cloisonner logiquement au sein d'un réseau support les UTL associées à des zones de niveaux de protection attendus distincts</t>
   </si>
   <si>
-    <t>Mutualisation des dispositifs de contrôle d'accès physique et de vidéoprotec- tion sur un même réseau support</t>
-  </si>
-  <si>
     <t>Éviter de mutualiser les dispositifs de contrôle d'accès et de vidéoprotection sur un même réseau support</t>
   </si>
   <si>
     <t>Mettre en place un cloisonnement logique entre les dispositifs de contrôle d'accès et de vidéoprotection mutualisés sur un même réseau support</t>
   </si>
   <si>
-    <t>Réseausupportdescamérasplacéesàl'extérieur de la zone contrôlée</t>
-  </si>
-  <si>
     <t>Dédier physiquement un réseau support pour les caméras extérieures</t>
   </si>
   <si>
     <t>Cloisonner logiquement le réseau des caméras extérieures</t>
   </si>
   <si>
-    <t>Réseaufédérateur</t>
-  </si>
-  <si>
     <t>Filtrage des flux entre les réseaux support</t>
   </si>
   <si>
@@ -1704,9 +1680,6 @@
     <t>Interconnexion</t>
   </si>
   <si>
-    <t>Interconnexionentreunsystèmedecontrôled'accèsphysiqueetleSIdel'entité</t>
-  </si>
-  <si>
     <t>Éviter une interconnexion avec le SI de l'entité</t>
   </si>
   <si>
@@ -1716,9 +1689,6 @@
     <t>Protéger les flux échangés entre le système de contrôle d'accès et le SI de l'entité</t>
   </si>
   <si>
-    <t>Interconnexion entre un système de contrôle d'accès physique et un système devidéoprotection</t>
-  </si>
-  <si>
     <t>Privilégier une solution s'appuyant sur deux centres de gestion distincts</t>
   </si>
   <si>
@@ -1737,9 +1707,6 @@
     <t>Sécurité des éléments support d'un système de contrôle d'accès physique</t>
   </si>
   <si>
-    <t>Badgesursupportphysique</t>
-  </si>
-  <si>
     <t>Ne pas stocker d'informations critiques sur le badge</t>
   </si>
   <si>
@@ -1755,9 +1722,6 @@
     <t>Garantir l'unicité d'un badge</t>
   </si>
   <si>
-    <t>Badgevirtuel sur ordiphone</t>
-  </si>
-  <si>
     <t>Éviter l'usage de badges virtuels sur ordiphone</t>
   </si>
   <si>
@@ -1944,9 +1908,6 @@
     <t>Anticiper la procédure de remplacement de clés cryptographiques en cas de compromission</t>
   </si>
   <si>
-    <t>Chiffrementetauthentificationdesfluxenprovenanceetàdestinationdesdispositifs devidéoprotection</t>
-  </si>
-  <si>
     <t>Privilégier les solutions d'authentification et de chiffrement non propriétaires</t>
   </si>
   <si>
@@ -2142,19 +2103,58 @@
     <t>Configurer des alertes en temps réel</t>
   </si>
   <si>
+    <t>[R] Recommandation à l'état de l'art</t>
+  </si>
+  <si>
+    <t>[R-] Recommandation alternative de premier niveau</t>
+  </si>
+  <si>
+    <t>[R+] Recommandation renforcée</t>
+  </si>
+  <si>
+    <t>ANSSI - Sécurisation des systèmes de contrôle d’accès physique et vidéoprotection (v2.2) [Recommandations]</t>
+  </si>
+  <si>
+    <t>Niveau de sûreté des équipements et des installations de contrôle d'accès physique</t>
+  </si>
+  <si>
+    <t>Connexions entre les têtes de lecture et l'UTL</t>
+  </si>
+  <si>
+    <t>Réseau support</t>
+  </si>
+  <si>
+    <t>Segmentation au sein du réseau support</t>
+  </si>
+  <si>
+    <t>Mutualisation des dispositifs de contrôle d'accès physique sur un même réseau support</t>
+  </si>
+  <si>
+    <t>Mutualisation des dispositifs de contrôle d'accès physique et de vidéoprotection sur un même réseau support</t>
+  </si>
+  <si>
+    <t>Réseau support des caméras placées à l'extérieur de la zone contrôlée</t>
+  </si>
+  <si>
+    <t>Réseau fédérateur</t>
+  </si>
+  <si>
+    <t>Interconnexion entre un système de contrôle d'accès physique et le SI de l'entité</t>
+  </si>
+  <si>
+    <t>Interconnexion entre un système de contrôle d'accès physique et un système de vidéoprotection</t>
+  </si>
+  <si>
+    <t>Badge sur support physique</t>
+  </si>
+  <si>
+    <t>Badge virtuel sur ordiphone</t>
+  </si>
+  <si>
+    <t>Chiffrement et authentification des flux en provenance et à destination des dispositifs de vidéoprotection</t>
+  </si>
+  <si>
     <t>Procéder immédiatement à l'interruption de l'alimentation électrique &amp; déconnexion du réseau support en cas de détection d'une tentative d'intrusion physique sur platine d'interphone ou visiophone IP.</t>
-  </si>
-  <si>
-    <t>[R] Recommandation à l'état de l'art</t>
-  </si>
-  <si>
-    <t>[R-] Recommandation alternative de premier niveau</t>
-  </si>
-  <si>
-    <t>[R+] Recommandation renforcée</t>
-  </si>
-  <si>
-    <t>ANSSI - Sécurisation des systèmes de contrôle d’accès physique et vidéoprotection (v2.2) [Recommandations]</t>
   </si>
 </sst>
 </file>
@@ -2588,7 +2588,7 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>696</v>
+        <v>682</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="302.39999999999998" x14ac:dyDescent="0.3">
@@ -2674,7 +2674,7 @@
         <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>696</v>
+        <v>682</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="273.60000000000002" x14ac:dyDescent="0.3">
@@ -2929,7 +2929,7 @@
         <v>52</v>
       </c>
       <c r="E13" t="s">
-        <v>497</v>
+        <v>683</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -2946,7 +2946,7 @@
         <v>54</v>
       </c>
       <c r="E14" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>55</v>
@@ -2963,7 +2963,7 @@
         <v>56</v>
       </c>
       <c r="E15" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
@@ -2980,7 +2980,7 @@
         <v>58</v>
       </c>
       <c r="E16" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>59</v>
@@ -2997,7 +2997,7 @@
         <v>60</v>
       </c>
       <c r="E17" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -3014,7 +3014,7 @@
         <v>62</v>
       </c>
       <c r="E18" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>63</v>
@@ -3031,7 +3031,7 @@
         <v>64</v>
       </c>
       <c r="E19" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -3048,7 +3048,7 @@
         <v>66</v>
       </c>
       <c r="E20" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>67</v>
@@ -3065,7 +3065,7 @@
         <v>68</v>
       </c>
       <c r="E21" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
@@ -3076,7 +3076,7 @@
         <v>69</v>
       </c>
       <c r="E22" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -3093,7 +3093,7 @@
         <v>71</v>
       </c>
       <c r="E23" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="F23" s="1" t="s">
         <v>72</v>
@@ -3116,7 +3116,7 @@
         <v>74</v>
       </c>
       <c r="E24" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>75</v>
@@ -3139,7 +3139,7 @@
         <v>78</v>
       </c>
       <c r="E25" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="F25" s="1" t="s">
         <v>79</v>
@@ -3156,7 +3156,7 @@
         <v>80</v>
       </c>
       <c r="E26" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
@@ -3167,7 +3167,7 @@
         <v>81</v>
       </c>
       <c r="E27" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -3184,7 +3184,7 @@
         <v>83</v>
       </c>
       <c r="E28" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>84</v>
@@ -3201,7 +3201,7 @@
         <v>85</v>
       </c>
       <c r="E29" t="s">
-        <v>513</v>
+        <v>684</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -3218,7 +3218,7 @@
         <v>87</v>
       </c>
       <c r="E30" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="F30" s="1" t="s">
         <v>88</v>
@@ -3241,7 +3241,7 @@
         <v>90</v>
       </c>
       <c r="E31" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="F31" s="1" t="s">
         <v>91</v>
@@ -3258,7 +3258,7 @@
         <v>92</v>
       </c>
       <c r="E32" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -3275,7 +3275,7 @@
         <v>94</v>
       </c>
       <c r="E33" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="F33" s="1" t="s">
         <v>95</v>
@@ -3298,7 +3298,7 @@
         <v>97</v>
       </c>
       <c r="E34" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="F34" s="1" t="s">
         <v>98</v>
@@ -3315,7 +3315,7 @@
         <v>99</v>
       </c>
       <c r="E35" t="s">
-        <v>519</v>
+        <v>685</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.3">
@@ -3326,7 +3326,7 @@
         <v>100</v>
       </c>
       <c r="E36" t="s">
-        <v>520</v>
+        <v>686</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -3343,7 +3343,7 @@
         <v>102</v>
       </c>
       <c r="E37" t="s">
-        <v>521</v>
+        <v>517</v>
       </c>
       <c r="F37" s="1" t="s">
         <v>103</v>
@@ -3360,7 +3360,7 @@
         <v>104</v>
       </c>
       <c r="E38" t="s">
-        <v>522</v>
+        <v>518</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -3377,7 +3377,7 @@
         <v>106</v>
       </c>
       <c r="E39" t="s">
-        <v>523</v>
+        <v>519</v>
       </c>
       <c r="F39" s="1" t="s">
         <v>107</v>
@@ -3400,7 +3400,7 @@
         <v>109</v>
       </c>
       <c r="E40" t="s">
-        <v>524</v>
+        <v>520</v>
       </c>
       <c r="F40" s="1" t="s">
         <v>110</v>
@@ -3423,7 +3423,7 @@
         <v>112</v>
       </c>
       <c r="E41" t="s">
-        <v>525</v>
+        <v>521</v>
       </c>
       <c r="F41" s="1" t="s">
         <v>113</v>
@@ -3446,7 +3446,7 @@
         <v>115</v>
       </c>
       <c r="E42" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="F42" s="1" t="s">
         <v>116</v>
@@ -3463,7 +3463,7 @@
         <v>117</v>
       </c>
       <c r="E43" t="s">
-        <v>527</v>
+        <v>687</v>
       </c>
     </row>
     <row r="44" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -3480,7 +3480,7 @@
         <v>119</v>
       </c>
       <c r="E44" t="s">
-        <v>528</v>
+        <v>523</v>
       </c>
       <c r="F44" s="1" t="s">
         <v>120</v>
@@ -3497,7 +3497,7 @@
         <v>121</v>
       </c>
       <c r="E45" t="s">
-        <v>529</v>
+        <v>688</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.3">
@@ -3514,7 +3514,7 @@
         <v>123</v>
       </c>
       <c r="E46" t="s">
-        <v>530</v>
+        <v>524</v>
       </c>
       <c r="F46" s="1" t="s">
         <v>124</v>
@@ -3537,7 +3537,7 @@
         <v>126</v>
       </c>
       <c r="E47" t="s">
-        <v>531</v>
+        <v>525</v>
       </c>
       <c r="F47" s="1" t="s">
         <v>127</v>
@@ -3557,7 +3557,7 @@
         <v>128</v>
       </c>
       <c r="E48" t="s">
-        <v>532</v>
+        <v>689</v>
       </c>
     </row>
     <row r="49" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -3574,7 +3574,7 @@
         <v>130</v>
       </c>
       <c r="E49" t="s">
-        <v>533</v>
+        <v>526</v>
       </c>
       <c r="F49" s="1" t="s">
         <v>131</v>
@@ -3597,7 +3597,7 @@
         <v>133</v>
       </c>
       <c r="E50" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="F50" s="1" t="s">
         <v>134</v>
@@ -3614,7 +3614,7 @@
         <v>135</v>
       </c>
       <c r="E51" t="s">
-        <v>535</v>
+        <v>690</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.3">
@@ -3625,7 +3625,7 @@
         <v>136</v>
       </c>
       <c r="E52" t="s">
-        <v>536</v>
+        <v>528</v>
       </c>
     </row>
     <row r="53" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -3642,7 +3642,7 @@
         <v>138</v>
       </c>
       <c r="E53" t="s">
-        <v>537</v>
+        <v>529</v>
       </c>
       <c r="F53" s="1" t="s">
         <v>139</v>
@@ -3659,7 +3659,7 @@
         <v>140</v>
       </c>
       <c r="E54" t="s">
-        <v>538</v>
+        <v>530</v>
       </c>
     </row>
     <row r="55" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
@@ -3676,7 +3676,7 @@
         <v>142</v>
       </c>
       <c r="E55" t="s">
-        <v>539</v>
+        <v>531</v>
       </c>
       <c r="F55" s="1" t="s">
         <v>479</v>
@@ -3693,7 +3693,7 @@
         <v>143</v>
       </c>
       <c r="E56" t="s">
-        <v>540</v>
+        <v>532</v>
       </c>
     </row>
     <row r="57" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -3710,7 +3710,7 @@
         <v>145</v>
       </c>
       <c r="E57" t="s">
-        <v>541</v>
+        <v>533</v>
       </c>
       <c r="F57" s="1" t="s">
         <v>146</v>
@@ -3727,7 +3727,7 @@
         <v>147</v>
       </c>
       <c r="E58" t="s">
-        <v>542</v>
+        <v>534</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.3">
@@ -3744,7 +3744,7 @@
         <v>149</v>
       </c>
       <c r="E59" t="s">
-        <v>543</v>
+        <v>535</v>
       </c>
       <c r="F59" s="1" t="s">
         <v>150</v>
@@ -3767,7 +3767,7 @@
         <v>152</v>
       </c>
       <c r="E60" t="s">
-        <v>544</v>
+        <v>536</v>
       </c>
       <c r="F60" s="1" t="s">
         <v>153</v>
@@ -3787,7 +3787,7 @@
         <v>154</v>
       </c>
       <c r="E61" t="s">
-        <v>545</v>
+        <v>537</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.3">
@@ -3798,7 +3798,7 @@
         <v>155</v>
       </c>
       <c r="E62" t="s">
-        <v>546</v>
+        <v>691</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.3">
@@ -3815,7 +3815,7 @@
         <v>157</v>
       </c>
       <c r="E63" t="s">
-        <v>547</v>
+        <v>538</v>
       </c>
       <c r="F63" s="1" t="s">
         <v>158</v>
@@ -3838,7 +3838,7 @@
         <v>160</v>
       </c>
       <c r="E64" t="s">
-        <v>548</v>
+        <v>539</v>
       </c>
       <c r="F64" s="1" t="s">
         <v>161</v>
@@ -3861,7 +3861,7 @@
         <v>163</v>
       </c>
       <c r="E65" t="s">
-        <v>549</v>
+        <v>540</v>
       </c>
       <c r="F65" s="1" t="s">
         <v>164</v>
@@ -3881,7 +3881,7 @@
         <v>165</v>
       </c>
       <c r="E66" t="s">
-        <v>550</v>
+        <v>692</v>
       </c>
     </row>
     <row r="67" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -3898,7 +3898,7 @@
         <v>167</v>
       </c>
       <c r="E67" t="s">
-        <v>551</v>
+        <v>541</v>
       </c>
       <c r="F67" s="1" t="s">
         <v>168</v>
@@ -3921,7 +3921,7 @@
         <v>170</v>
       </c>
       <c r="E68" t="s">
-        <v>552</v>
+        <v>542</v>
       </c>
       <c r="F68" s="1" t="s">
         <v>171</v>
@@ -3938,7 +3938,7 @@
         <v>172</v>
       </c>
       <c r="E69" t="s">
-        <v>553</v>
+        <v>543</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.3">
@@ -3949,7 +3949,7 @@
         <v>173</v>
       </c>
       <c r="E70" t="s">
-        <v>554</v>
+        <v>544</v>
       </c>
     </row>
     <row r="71" spans="1:8" ht="158.4" x14ac:dyDescent="0.3">
@@ -3966,7 +3966,7 @@
         <v>175</v>
       </c>
       <c r="E71" t="s">
-        <v>555</v>
+        <v>545</v>
       </c>
       <c r="F71" s="1" t="s">
         <v>480</v>
@@ -3983,7 +3983,7 @@
         <v>176</v>
       </c>
       <c r="E72" t="s">
-        <v>556</v>
+        <v>546</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.3">
@@ -3994,7 +3994,7 @@
         <v>177</v>
       </c>
       <c r="E73" t="s">
-        <v>557</v>
+        <v>693</v>
       </c>
     </row>
     <row r="74" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
@@ -4011,7 +4011,7 @@
         <v>179</v>
       </c>
       <c r="E74" t="s">
-        <v>558</v>
+        <v>547</v>
       </c>
       <c r="F74" s="1" t="s">
         <v>180</v>
@@ -4037,7 +4037,7 @@
         <v>182</v>
       </c>
       <c r="E75" t="s">
-        <v>559</v>
+        <v>548</v>
       </c>
       <c r="F75" s="1" t="s">
         <v>183</v>
@@ -4060,7 +4060,7 @@
         <v>185</v>
       </c>
       <c r="E76" t="s">
-        <v>560</v>
+        <v>549</v>
       </c>
       <c r="F76" s="1" t="s">
         <v>481</v>
@@ -4083,7 +4083,7 @@
         <v>187</v>
       </c>
       <c r="E77" t="s">
-        <v>561</v>
+        <v>550</v>
       </c>
       <c r="F77" s="1" t="s">
         <v>188</v>
@@ -4106,7 +4106,7 @@
         <v>190</v>
       </c>
       <c r="E78" t="s">
-        <v>562</v>
+        <v>551</v>
       </c>
       <c r="F78" s="1" t="s">
         <v>191</v>
@@ -4123,7 +4123,7 @@
         <v>192</v>
       </c>
       <c r="E79" t="s">
-        <v>563</v>
+        <v>694</v>
       </c>
     </row>
     <row r="80" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -4140,7 +4140,7 @@
         <v>194</v>
       </c>
       <c r="E80" t="s">
-        <v>564</v>
+        <v>552</v>
       </c>
       <c r="F80" s="1" t="s">
         <v>195</v>
@@ -4157,7 +4157,7 @@
         <v>196</v>
       </c>
       <c r="E81" t="s">
-        <v>565</v>
+        <v>553</v>
       </c>
     </row>
     <row r="82" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -4174,7 +4174,7 @@
         <v>198</v>
       </c>
       <c r="E82" t="s">
-        <v>566</v>
+        <v>554</v>
       </c>
       <c r="F82" s="1" t="s">
         <v>199</v>
@@ -4197,7 +4197,7 @@
         <v>201</v>
       </c>
       <c r="E83" t="s">
-        <v>567</v>
+        <v>555</v>
       </c>
       <c r="F83" s="1" t="s">
         <v>202</v>
@@ -4214,7 +4214,7 @@
         <v>203</v>
       </c>
       <c r="E84" t="s">
-        <v>568</v>
+        <v>556</v>
       </c>
     </row>
     <row r="85" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -4231,7 +4231,7 @@
         <v>205</v>
       </c>
       <c r="E85" t="s">
-        <v>569</v>
+        <v>557</v>
       </c>
       <c r="F85" s="1" t="s">
         <v>206</v>
@@ -4254,7 +4254,7 @@
         <v>208</v>
       </c>
       <c r="E86" t="s">
-        <v>570</v>
+        <v>558</v>
       </c>
       <c r="F86" s="1" t="s">
         <v>209</v>
@@ -4277,7 +4277,7 @@
         <v>211</v>
       </c>
       <c r="E87" t="s">
-        <v>571</v>
+        <v>559</v>
       </c>
       <c r="F87" s="1" t="s">
         <v>212</v>
@@ -4294,7 +4294,7 @@
         <v>213</v>
       </c>
       <c r="E88" t="s">
-        <v>572</v>
+        <v>560</v>
       </c>
     </row>
     <row r="89" spans="1:8" ht="72" x14ac:dyDescent="0.3">
@@ -4311,7 +4311,7 @@
         <v>215</v>
       </c>
       <c r="E89" t="s">
-        <v>573</v>
+        <v>561</v>
       </c>
       <c r="F89" s="1" t="s">
         <v>216</v>
@@ -4328,7 +4328,7 @@
         <v>217</v>
       </c>
       <c r="E90" t="s">
-        <v>574</v>
+        <v>562</v>
       </c>
     </row>
     <row r="91" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -4345,7 +4345,7 @@
         <v>219</v>
       </c>
       <c r="E91" t="s">
-        <v>575</v>
+        <v>563</v>
       </c>
       <c r="F91" s="1" t="s">
         <v>220</v>
@@ -4362,7 +4362,7 @@
         <v>221</v>
       </c>
       <c r="E92" t="s">
-        <v>576</v>
+        <v>564</v>
       </c>
     </row>
     <row r="93" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -4379,7 +4379,7 @@
         <v>223</v>
       </c>
       <c r="E93" t="s">
-        <v>577</v>
+        <v>565</v>
       </c>
       <c r="F93" s="1" t="s">
         <v>224</v>
@@ -4402,7 +4402,7 @@
         <v>226</v>
       </c>
       <c r="E94" t="s">
-        <v>578</v>
+        <v>566</v>
       </c>
       <c r="F94" s="1" t="s">
         <v>227</v>
@@ -4419,7 +4419,7 @@
         <v>228</v>
       </c>
       <c r="E95" t="s">
-        <v>579</v>
+        <v>567</v>
       </c>
     </row>
     <row r="96" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -4436,7 +4436,7 @@
         <v>230</v>
       </c>
       <c r="E96" t="s">
-        <v>580</v>
+        <v>568</v>
       </c>
       <c r="F96" s="1" t="s">
         <v>231</v>
@@ -4459,7 +4459,7 @@
         <v>233</v>
       </c>
       <c r="E97" t="s">
-        <v>581</v>
+        <v>569</v>
       </c>
       <c r="F97" s="1" t="s">
         <v>234</v>
@@ -4482,7 +4482,7 @@
         <v>237</v>
       </c>
       <c r="E98" t="s">
-        <v>582</v>
+        <v>570</v>
       </c>
       <c r="F98" s="1" t="s">
         <v>238</v>
@@ -4508,7 +4508,7 @@
         <v>240</v>
       </c>
       <c r="E99" t="s">
-        <v>583</v>
+        <v>571</v>
       </c>
       <c r="F99" s="1" t="s">
         <v>241</v>
@@ -4531,7 +4531,7 @@
         <v>243</v>
       </c>
       <c r="E100" t="s">
-        <v>692</v>
+        <v>696</v>
       </c>
       <c r="F100" s="1" t="s">
         <v>244</v>
@@ -4554,7 +4554,7 @@
         <v>246</v>
       </c>
       <c r="E101" t="s">
-        <v>584</v>
+        <v>572</v>
       </c>
       <c r="F101" s="1" t="s">
         <v>247</v>
@@ -4571,7 +4571,7 @@
         <v>248</v>
       </c>
       <c r="E102" t="s">
-        <v>585</v>
+        <v>573</v>
       </c>
     </row>
     <row r="103" spans="1:8" x14ac:dyDescent="0.3">
@@ -4582,7 +4582,7 @@
         <v>249</v>
       </c>
       <c r="E103" t="s">
-        <v>586</v>
+        <v>574</v>
       </c>
     </row>
     <row r="104" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -4599,7 +4599,7 @@
         <v>251</v>
       </c>
       <c r="E104" t="s">
-        <v>587</v>
+        <v>575</v>
       </c>
       <c r="F104" s="1" t="s">
         <v>252</v>
@@ -4622,7 +4622,7 @@
         <v>254</v>
       </c>
       <c r="E105" t="s">
-        <v>588</v>
+        <v>576</v>
       </c>
       <c r="F105" s="1" t="s">
         <v>255</v>
@@ -4645,7 +4645,7 @@
         <v>257</v>
       </c>
       <c r="E106" t="s">
-        <v>589</v>
+        <v>577</v>
       </c>
       <c r="F106" s="1" t="s">
         <v>258</v>
@@ -4668,7 +4668,7 @@
         <v>260</v>
       </c>
       <c r="E107" t="s">
-        <v>590</v>
+        <v>578</v>
       </c>
       <c r="F107" s="1" t="s">
         <v>261</v>
@@ -4691,7 +4691,7 @@
         <v>263</v>
       </c>
       <c r="E108" t="s">
-        <v>591</v>
+        <v>579</v>
       </c>
       <c r="F108" s="1" t="s">
         <v>264</v>
@@ -4714,7 +4714,7 @@
         <v>266</v>
       </c>
       <c r="E109" t="s">
-        <v>592</v>
+        <v>580</v>
       </c>
       <c r="F109" s="1" t="s">
         <v>482</v>
@@ -4731,7 +4731,7 @@
         <v>267</v>
       </c>
       <c r="E110" t="s">
-        <v>593</v>
+        <v>581</v>
       </c>
     </row>
     <row r="111" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -4748,7 +4748,7 @@
         <v>269</v>
       </c>
       <c r="E111" t="s">
-        <v>594</v>
+        <v>582</v>
       </c>
       <c r="F111" s="1" t="s">
         <v>270</v>
@@ -4771,7 +4771,7 @@
         <v>272</v>
       </c>
       <c r="E112" t="s">
-        <v>595</v>
+        <v>583</v>
       </c>
       <c r="F112" s="1" t="s">
         <v>273</v>
@@ -4794,7 +4794,7 @@
         <v>275</v>
       </c>
       <c r="E113" t="s">
-        <v>596</v>
+        <v>584</v>
       </c>
       <c r="F113" s="1" t="s">
         <v>276</v>
@@ -4820,7 +4820,7 @@
         <v>278</v>
       </c>
       <c r="E114" t="s">
-        <v>597</v>
+        <v>585</v>
       </c>
       <c r="F114" s="1" t="s">
         <v>279</v>
@@ -4843,7 +4843,7 @@
         <v>281</v>
       </c>
       <c r="E115" t="s">
-        <v>598</v>
+        <v>586</v>
       </c>
       <c r="F115" s="1" t="s">
         <v>282</v>
@@ -4866,7 +4866,7 @@
         <v>284</v>
       </c>
       <c r="E116" t="s">
-        <v>599</v>
+        <v>587</v>
       </c>
       <c r="F116" s="1" t="s">
         <v>285</v>
@@ -4889,7 +4889,7 @@
         <v>287</v>
       </c>
       <c r="E117" t="s">
-        <v>600</v>
+        <v>588</v>
       </c>
       <c r="F117" s="1" t="s">
         <v>288</v>
@@ -4906,7 +4906,7 @@
         <v>289</v>
       </c>
       <c r="E118" t="s">
-        <v>601</v>
+        <v>589</v>
       </c>
     </row>
     <row r="119" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -4923,7 +4923,7 @@
         <v>291</v>
       </c>
       <c r="E119" t="s">
-        <v>602</v>
+        <v>590</v>
       </c>
       <c r="F119" s="1" t="s">
         <v>292</v>
@@ -4940,7 +4940,7 @@
         <v>293</v>
       </c>
       <c r="E120" t="s">
-        <v>603</v>
+        <v>591</v>
       </c>
     </row>
     <row r="121" spans="1:8" x14ac:dyDescent="0.3">
@@ -4951,7 +4951,7 @@
         <v>294</v>
       </c>
       <c r="E121" t="s">
-        <v>604</v>
+        <v>592</v>
       </c>
     </row>
     <row r="122" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -4968,7 +4968,7 @@
         <v>296</v>
       </c>
       <c r="E122" t="s">
-        <v>605</v>
+        <v>593</v>
       </c>
       <c r="F122" s="1" t="s">
         <v>297</v>
@@ -4985,7 +4985,7 @@
         <v>298</v>
       </c>
       <c r="E123" t="s">
-        <v>606</v>
+        <v>594</v>
       </c>
     </row>
     <row r="124" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -5002,7 +5002,7 @@
         <v>300</v>
       </c>
       <c r="E124" t="s">
-        <v>607</v>
+        <v>595</v>
       </c>
       <c r="F124" s="1" t="s">
         <v>301</v>
@@ -5019,7 +5019,7 @@
         <v>302</v>
       </c>
       <c r="E125" t="s">
-        <v>608</v>
+        <v>596</v>
       </c>
     </row>
     <row r="126" spans="1:8" ht="72" x14ac:dyDescent="0.3">
@@ -5036,7 +5036,7 @@
         <v>304</v>
       </c>
       <c r="E126" t="s">
-        <v>609</v>
+        <v>597</v>
       </c>
       <c r="F126" s="1" t="s">
         <v>305</v>
@@ -5059,7 +5059,7 @@
         <v>307</v>
       </c>
       <c r="E127" t="s">
-        <v>610</v>
+        <v>598</v>
       </c>
       <c r="F127" s="1" t="s">
         <v>308</v>
@@ -5076,7 +5076,7 @@
         <v>309</v>
       </c>
       <c r="E128" t="s">
-        <v>611</v>
+        <v>599</v>
       </c>
     </row>
     <row r="129" spans="1:8" x14ac:dyDescent="0.3">
@@ -5087,7 +5087,7 @@
         <v>310</v>
       </c>
       <c r="E129" t="s">
-        <v>612</v>
+        <v>600</v>
       </c>
     </row>
     <row r="130" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -5104,7 +5104,7 @@
         <v>312</v>
       </c>
       <c r="E130" t="s">
-        <v>613</v>
+        <v>601</v>
       </c>
       <c r="F130" s="1" t="s">
         <v>313</v>
@@ -5121,7 +5121,7 @@
         <v>314</v>
       </c>
       <c r="E131" t="s">
-        <v>614</v>
+        <v>602</v>
       </c>
     </row>
     <row r="132" spans="1:8" x14ac:dyDescent="0.3">
@@ -5138,7 +5138,7 @@
         <v>316</v>
       </c>
       <c r="E132" t="s">
-        <v>615</v>
+        <v>603</v>
       </c>
       <c r="F132" s="1" t="s">
         <v>317</v>
@@ -5161,7 +5161,7 @@
         <v>319</v>
       </c>
       <c r="E133" t="s">
-        <v>616</v>
+        <v>604</v>
       </c>
       <c r="F133" s="1" t="s">
         <v>320</v>
@@ -5178,7 +5178,7 @@
         <v>321</v>
       </c>
       <c r="E134" t="s">
-        <v>617</v>
+        <v>605</v>
       </c>
     </row>
     <row r="135" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -5195,7 +5195,7 @@
         <v>323</v>
       </c>
       <c r="E135" t="s">
-        <v>618</v>
+        <v>606</v>
       </c>
       <c r="F135" s="1" t="s">
         <v>324</v>
@@ -5218,7 +5218,7 @@
         <v>326</v>
       </c>
       <c r="E136" t="s">
-        <v>619</v>
+        <v>607</v>
       </c>
       <c r="F136" s="1" t="s">
         <v>327</v>
@@ -5235,7 +5235,7 @@
         <v>328</v>
       </c>
       <c r="E137" t="s">
-        <v>620</v>
+        <v>608</v>
       </c>
     </row>
     <row r="138" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -5252,7 +5252,7 @@
         <v>330</v>
       </c>
       <c r="E138" t="s">
-        <v>621</v>
+        <v>609</v>
       </c>
       <c r="F138" s="1" t="s">
         <v>331</v>
@@ -5269,7 +5269,7 @@
         <v>332</v>
       </c>
       <c r="E139" t="s">
-        <v>622</v>
+        <v>610</v>
       </c>
     </row>
     <row r="140" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -5286,7 +5286,7 @@
         <v>334</v>
       </c>
       <c r="E140" t="s">
-        <v>623</v>
+        <v>611</v>
       </c>
       <c r="F140" s="1" t="s">
         <v>335</v>
@@ -5309,7 +5309,7 @@
         <v>337</v>
       </c>
       <c r="E141" t="s">
-        <v>624</v>
+        <v>612</v>
       </c>
       <c r="F141" s="1" t="s">
         <v>338</v>
@@ -5332,7 +5332,7 @@
         <v>340</v>
       </c>
       <c r="E142" t="s">
-        <v>625</v>
+        <v>613</v>
       </c>
       <c r="F142" s="1" t="s">
         <v>341</v>
@@ -5349,7 +5349,7 @@
         <v>342</v>
       </c>
       <c r="E143" t="s">
-        <v>626</v>
+        <v>695</v>
       </c>
     </row>
     <row r="144" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -5366,7 +5366,7 @@
         <v>344</v>
       </c>
       <c r="E144" t="s">
-        <v>627</v>
+        <v>614</v>
       </c>
       <c r="F144" s="1" t="s">
         <v>345</v>
@@ -5383,7 +5383,7 @@
         <v>346</v>
       </c>
       <c r="E145" t="s">
-        <v>628</v>
+        <v>615</v>
       </c>
     </row>
     <row r="146" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
@@ -5400,7 +5400,7 @@
         <v>348</v>
       </c>
       <c r="E146" t="s">
-        <v>629</v>
+        <v>616</v>
       </c>
       <c r="F146" s="1" t="s">
         <v>349</v>
@@ -5417,7 +5417,7 @@
         <v>350</v>
       </c>
       <c r="E147" t="s">
-        <v>630</v>
+        <v>617</v>
       </c>
     </row>
     <row r="148" spans="1:8" x14ac:dyDescent="0.3">
@@ -5428,7 +5428,7 @@
         <v>351</v>
       </c>
       <c r="E148" t="s">
-        <v>631</v>
+        <v>618</v>
       </c>
     </row>
     <row r="149" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -5445,7 +5445,7 @@
         <v>353</v>
       </c>
       <c r="E149" t="s">
-        <v>632</v>
+        <v>619</v>
       </c>
       <c r="F149" s="1" t="s">
         <v>354</v>
@@ -5462,7 +5462,7 @@
         <v>355</v>
       </c>
       <c r="E150" t="s">
-        <v>633</v>
+        <v>620</v>
       </c>
     </row>
     <row r="151" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -5479,7 +5479,7 @@
         <v>357</v>
       </c>
       <c r="E151" t="s">
-        <v>634</v>
+        <v>621</v>
       </c>
       <c r="F151" s="1" t="s">
         <v>358</v>
@@ -5496,7 +5496,7 @@
         <v>359</v>
       </c>
       <c r="E152" t="s">
-        <v>635</v>
+        <v>622</v>
       </c>
     </row>
     <row r="153" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -5513,7 +5513,7 @@
         <v>361</v>
       </c>
       <c r="E153" t="s">
-        <v>636</v>
+        <v>623</v>
       </c>
       <c r="F153" s="1" t="s">
         <v>362</v>
@@ -5536,7 +5536,7 @@
         <v>364</v>
       </c>
       <c r="E154" t="s">
-        <v>637</v>
+        <v>624</v>
       </c>
       <c r="F154" s="1" t="s">
         <v>365</v>
@@ -5553,7 +5553,7 @@
         <v>366</v>
       </c>
       <c r="E155" t="s">
-        <v>638</v>
+        <v>625</v>
       </c>
     </row>
     <row r="156" spans="1:8" x14ac:dyDescent="0.3">
@@ -5564,7 +5564,7 @@
         <v>367</v>
       </c>
       <c r="E156" t="s">
-        <v>639</v>
+        <v>626</v>
       </c>
     </row>
     <row r="157" spans="1:8" x14ac:dyDescent="0.3">
@@ -5575,7 +5575,7 @@
         <v>368</v>
       </c>
       <c r="E157" t="s">
-        <v>640</v>
+        <v>627</v>
       </c>
     </row>
     <row r="158" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -5592,7 +5592,7 @@
         <v>370</v>
       </c>
       <c r="E158" t="s">
-        <v>641</v>
+        <v>628</v>
       </c>
       <c r="F158" s="1" t="s">
         <v>371</v>
@@ -5615,7 +5615,7 @@
         <v>373</v>
       </c>
       <c r="E159" t="s">
-        <v>642</v>
+        <v>629</v>
       </c>
       <c r="F159" s="1" t="s">
         <v>374</v>
@@ -5632,7 +5632,7 @@
         <v>375</v>
       </c>
       <c r="E160" t="s">
-        <v>643</v>
+        <v>630</v>
       </c>
     </row>
     <row r="161" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -5649,7 +5649,7 @@
         <v>377</v>
       </c>
       <c r="E161" t="s">
-        <v>644</v>
+        <v>631</v>
       </c>
       <c r="F161" s="1" t="s">
         <v>378</v>
@@ -5666,7 +5666,7 @@
         <v>379</v>
       </c>
       <c r="E162" t="s">
-        <v>645</v>
+        <v>632</v>
       </c>
     </row>
     <row r="163" spans="1:8" x14ac:dyDescent="0.3">
@@ -5677,7 +5677,7 @@
         <v>380</v>
       </c>
       <c r="E163" t="s">
-        <v>646</v>
+        <v>633</v>
       </c>
     </row>
     <row r="164" spans="1:8" ht="72" x14ac:dyDescent="0.3">
@@ -5694,7 +5694,7 @@
         <v>382</v>
       </c>
       <c r="E164" t="s">
-        <v>647</v>
+        <v>634</v>
       </c>
       <c r="F164" s="1" t="s">
         <v>483</v>
@@ -5711,7 +5711,7 @@
         <v>383</v>
       </c>
       <c r="E165" t="s">
-        <v>648</v>
+        <v>635</v>
       </c>
     </row>
     <row r="166" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -5728,7 +5728,7 @@
         <v>385</v>
       </c>
       <c r="E166" t="s">
-        <v>649</v>
+        <v>636</v>
       </c>
       <c r="F166" s="1" t="s">
         <v>386</v>
@@ -5745,7 +5745,7 @@
         <v>387</v>
       </c>
       <c r="E167" t="s">
-        <v>650</v>
+        <v>637</v>
       </c>
     </row>
     <row r="168" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -5762,7 +5762,7 @@
         <v>389</v>
       </c>
       <c r="E168" t="s">
-        <v>651</v>
+        <v>638</v>
       </c>
       <c r="F168" s="1" t="s">
         <v>390</v>
@@ -5779,7 +5779,7 @@
         <v>391</v>
       </c>
       <c r="E169" t="s">
-        <v>652</v>
+        <v>639</v>
       </c>
     </row>
     <row r="170" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -5796,7 +5796,7 @@
         <v>393</v>
       </c>
       <c r="E170" t="s">
-        <v>653</v>
+        <v>640</v>
       </c>
       <c r="F170" s="1" t="s">
         <v>394</v>
@@ -5813,7 +5813,7 @@
         <v>395</v>
       </c>
       <c r="E171" t="s">
-        <v>654</v>
+        <v>641</v>
       </c>
     </row>
     <row r="172" spans="1:8" x14ac:dyDescent="0.3">
@@ -5824,7 +5824,7 @@
         <v>396</v>
       </c>
       <c r="E172" t="s">
-        <v>655</v>
+        <v>642</v>
       </c>
     </row>
     <row r="173" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -5841,7 +5841,7 @@
         <v>398</v>
       </c>
       <c r="E173" t="s">
-        <v>656</v>
+        <v>643</v>
       </c>
       <c r="F173" s="1" t="s">
         <v>399</v>
@@ -5858,7 +5858,7 @@
         <v>400</v>
       </c>
       <c r="E174" t="s">
-        <v>657</v>
+        <v>644</v>
       </c>
     </row>
     <row r="175" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
@@ -5875,7 +5875,7 @@
         <v>402</v>
       </c>
       <c r="E175" t="s">
-        <v>658</v>
+        <v>645</v>
       </c>
       <c r="F175" s="1" t="s">
         <v>484</v>
@@ -5892,7 +5892,7 @@
         <v>403</v>
       </c>
       <c r="E176" t="s">
-        <v>659</v>
+        <v>646</v>
       </c>
     </row>
     <row r="177" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -5909,7 +5909,7 @@
         <v>405</v>
       </c>
       <c r="E177" t="s">
-        <v>660</v>
+        <v>647</v>
       </c>
       <c r="F177" s="1" t="s">
         <v>406</v>
@@ -5932,7 +5932,7 @@
         <v>408</v>
       </c>
       <c r="E178" t="s">
-        <v>661</v>
+        <v>648</v>
       </c>
       <c r="F178" s="1" t="s">
         <v>409</v>
@@ -5955,7 +5955,7 @@
         <v>411</v>
       </c>
       <c r="E179" t="s">
-        <v>662</v>
+        <v>649</v>
       </c>
       <c r="F179" s="1" t="s">
         <v>412</v>
@@ -5972,7 +5972,7 @@
         <v>413</v>
       </c>
       <c r="E180" t="s">
-        <v>663</v>
+        <v>650</v>
       </c>
     </row>
     <row r="181" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -5989,7 +5989,7 @@
         <v>415</v>
       </c>
       <c r="E181" t="s">
-        <v>664</v>
+        <v>651</v>
       </c>
       <c r="F181" s="1" t="s">
         <v>416</v>
@@ -6006,7 +6006,7 @@
         <v>417</v>
       </c>
       <c r="E182" t="s">
-        <v>665</v>
+        <v>652</v>
       </c>
     </row>
     <row r="183" spans="1:8" x14ac:dyDescent="0.3">
@@ -6017,7 +6017,7 @@
         <v>418</v>
       </c>
       <c r="E183" t="s">
-        <v>666</v>
+        <v>653</v>
       </c>
     </row>
     <row r="184" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -6034,7 +6034,7 @@
         <v>420</v>
       </c>
       <c r="E184" t="s">
-        <v>667</v>
+        <v>654</v>
       </c>
       <c r="F184" s="1" t="s">
         <v>421</v>
@@ -6057,7 +6057,7 @@
         <v>423</v>
       </c>
       <c r="E185" t="s">
-        <v>668</v>
+        <v>655</v>
       </c>
       <c r="F185" s="1" t="s">
         <v>424</v>
@@ -6080,7 +6080,7 @@
         <v>426</v>
       </c>
       <c r="E186" t="s">
-        <v>669</v>
+        <v>656</v>
       </c>
       <c r="F186" s="1" t="s">
         <v>427</v>
@@ -6097,7 +6097,7 @@
         <v>428</v>
       </c>
       <c r="E187" t="s">
-        <v>670</v>
+        <v>657</v>
       </c>
     </row>
     <row r="188" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -6114,7 +6114,7 @@
         <v>430</v>
       </c>
       <c r="E188" t="s">
-        <v>671</v>
+        <v>658</v>
       </c>
       <c r="F188" s="1" t="s">
         <v>431</v>
@@ -6131,7 +6131,7 @@
         <v>432</v>
       </c>
       <c r="E189" t="s">
-        <v>672</v>
+        <v>659</v>
       </c>
     </row>
     <row r="190" spans="1:8" x14ac:dyDescent="0.3">
@@ -6142,7 +6142,7 @@
         <v>433</v>
       </c>
       <c r="E190" t="s">
-        <v>673</v>
+        <v>660</v>
       </c>
     </row>
     <row r="191" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -6159,7 +6159,7 @@
         <v>435</v>
       </c>
       <c r="E191" t="s">
-        <v>674</v>
+        <v>661</v>
       </c>
       <c r="F191" s="1" t="s">
         <v>436</v>
@@ -6176,7 +6176,7 @@
         <v>437</v>
       </c>
       <c r="E192" t="s">
-        <v>675</v>
+        <v>662</v>
       </c>
     </row>
     <row r="193" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -6193,7 +6193,7 @@
         <v>439</v>
       </c>
       <c r="E193" t="s">
-        <v>676</v>
+        <v>663</v>
       </c>
       <c r="F193" s="1" t="s">
         <v>485</v>
@@ -6210,7 +6210,7 @@
         <v>440</v>
       </c>
       <c r="E194" t="s">
-        <v>677</v>
+        <v>664</v>
       </c>
     </row>
     <row r="195" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -6227,7 +6227,7 @@
         <v>442</v>
       </c>
       <c r="E195" t="s">
-        <v>678</v>
+        <v>665</v>
       </c>
       <c r="F195" s="1" t="s">
         <v>443</v>
@@ -6244,7 +6244,7 @@
         <v>444</v>
       </c>
       <c r="E196" t="s">
-        <v>679</v>
+        <v>666</v>
       </c>
     </row>
     <row r="197" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
@@ -6261,7 +6261,7 @@
         <v>446</v>
       </c>
       <c r="E197" t="s">
-        <v>680</v>
+        <v>667</v>
       </c>
       <c r="F197" s="1" t="s">
         <v>447</v>
@@ -6278,7 +6278,7 @@
         <v>448</v>
       </c>
       <c r="E198" t="s">
-        <v>681</v>
+        <v>668</v>
       </c>
     </row>
     <row r="199" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -6295,7 +6295,7 @@
         <v>450</v>
       </c>
       <c r="E199" t="s">
-        <v>682</v>
+        <v>669</v>
       </c>
       <c r="F199" s="1" t="s">
         <v>451</v>
@@ -6312,7 +6312,7 @@
         <v>452</v>
       </c>
       <c r="E200" t="s">
-        <v>683</v>
+        <v>670</v>
       </c>
     </row>
     <row r="201" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -6329,7 +6329,7 @@
         <v>454</v>
       </c>
       <c r="E201" t="s">
-        <v>684</v>
+        <v>671</v>
       </c>
       <c r="F201" s="1" t="s">
         <v>455</v>
@@ -6346,7 +6346,7 @@
         <v>456</v>
       </c>
       <c r="E202" t="s">
-        <v>685</v>
+        <v>672</v>
       </c>
     </row>
     <row r="203" spans="1:8" x14ac:dyDescent="0.3">
@@ -6357,7 +6357,7 @@
         <v>457</v>
       </c>
       <c r="E203" t="s">
-        <v>686</v>
+        <v>673</v>
       </c>
     </row>
     <row r="204" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -6374,7 +6374,7 @@
         <v>459</v>
       </c>
       <c r="E204" t="s">
-        <v>687</v>
+        <v>674</v>
       </c>
       <c r="F204" s="1" t="s">
         <v>460</v>
@@ -6391,7 +6391,7 @@
         <v>461</v>
       </c>
       <c r="E205" t="s">
-        <v>688</v>
+        <v>675</v>
       </c>
     </row>
     <row r="206" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -6408,7 +6408,7 @@
         <v>463</v>
       </c>
       <c r="E206" t="s">
-        <v>689</v>
+        <v>676</v>
       </c>
       <c r="F206" s="1" t="s">
         <v>464</v>
@@ -6425,7 +6425,7 @@
         <v>465</v>
       </c>
       <c r="E207" t="s">
-        <v>690</v>
+        <v>677</v>
       </c>
     </row>
     <row r="208" spans="1:8" x14ac:dyDescent="0.3">
@@ -6442,7 +6442,7 @@
         <v>467</v>
       </c>
       <c r="E208" t="s">
-        <v>691</v>
+        <v>678</v>
       </c>
       <c r="F208" s="1" t="s">
         <v>468</v>
@@ -6513,7 +6513,7 @@
         <v>36</v>
       </c>
       <c r="B2" t="s">
-        <v>693</v>
+        <v>679</v>
       </c>
       <c r="C2" t="s">
         <v>469</v>
@@ -6524,7 +6524,7 @@
         <v>76</v>
       </c>
       <c r="B3" t="s">
-        <v>694</v>
+        <v>680</v>
       </c>
       <c r="C3" t="s">
         <v>470</v>
@@ -6535,7 +6535,7 @@
         <v>235</v>
       </c>
       <c r="B4" t="s">
-        <v>695</v>
+        <v>681</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>471</v>

</xml_diff>

<commit_message>
Fix 2 Framework section Names (YAML + Excel + Script)
</commit_message>
<xml_diff>
--- a/tools/excel/anssi/rec-secu-sys-ctrl-acces-phys-videoprot/anssi_rec-secu-sys-ctrl-acces-phys-videoprot_v2.2.xlsx
+++ b/tools/excel/anssi/rec-secu-sys-ctrl-acces-phys-videoprot/anssi_rec-secu-sys-ctrl-acces-phys-videoprot_v2.2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\tarkadia\projects\intuitem\ciso-assistant-community\tools\excel\anssi\rec-secu-sys-ctrl-acces-phys-videoprot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E0AF98F-EBAB-4246-A1FA-3AF806A060D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9317182-A9DF-4153-9DC2-843CE2184AA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1485" yWindow="-15870" windowWidth="25440" windowHeight="15990" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1845" yWindow="-14055" windowWidth="19710" windowHeight="12330" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="library_meta" sheetId="1" r:id="rId1"/>
@@ -1496,12 +1496,6 @@
 * document répertoriant les périmètres et niveaux de privilèges des utilisateurs et des administrateurs.</t>
   </si>
   <si>
-    <t>Il est recommandé que les badges soient visuellement les plus neutres possibles. Ils ne doivent notamment pas indiquer:
-* d'informations sur l'entreprise (nom, adresse) &lt;abbr title="Si des coordonnées sont indiquées sur le dos du badge pour faciliter sa restitution en cas de perte, elles ne doivent pas mentionner explicitement le nom de l&amp;#x27;entité. Mieux vaut privilégier dans ce cas l&amp;#x27;utilisation d&amp;#x27;une boîte postale."&gt;&lt;sup&gt;24&lt;/sup&gt;&lt;/abbr&gt;;
-* d'informations sur le porteur (nom, prénom, poste), en dehors de sa photo;
-* les accès autorisés. Un numéro de traçabilité peut être indiqué sur le badge à des fins administratives, mais ce numéro doit être différent du numéro d'identification. La photographie est tolérée car elle permet de vérifier rapidement que le badge appartient bien au porteur. XXXX La puce contient l'UID et le numéro d'identification YYYY Concernant les types de badges, les supports de type puce RFID &lt;abbr title="Radio Frequency Identification."&gt;&lt;sup&gt;25&lt;/sup&gt;&lt;/abbr&gt;, comparables aux antivols dans les magasins, ne permettent que l'identification, tandis que les supports de type carte à puce, comparables aux cartes de paiement bancaire, disposent de fonctions cryptographiques qui permettent une authentification. Certaines technologies de carte d'accès, qui font appel à des mécanismes cryptographiques faibles, ont des vulnérabilités connues qui permettent leur clonage et des attaques par rejeu &lt;abbr title="Attaque dans laquelle une transmission est frauduleusement répétée par une tierce partie interceptant les paquets sur la ligne."&gt;&lt;sup&gt;26&lt;/sup&gt;&lt;/abbr&gt;. Il convient donc de s'orienter vers des produits récents, dont le niveau de sécurité est satisfaisant à date et dont le protocole de communication et la fonction anti-clone sont résistants à des attaques de niveau AV A_V AN.327.</t>
-  </si>
-  <si>
     <t>Il est recommandé d'adopter une approche prudente et sélective concernant l'installation d'applications sur les caméras de surveillance. Pour cela:
 * désactiver systématiquement les fonctionnalités non essentielles au déploiement spécifique;
 * limiter les installations aux seules applications répondant aux besoins opérationnels de l'entreprise.</t>
@@ -2155,6 +2149,12 @@
   </si>
   <si>
     <t>Procéder immédiatement à l'interruption de l'alimentation électrique &amp; déconnexion du réseau support en cas de détection d'une tentative d'intrusion physique sur platine d'interphone ou visiophone IP.</t>
+  </si>
+  <si>
+    <t>Il est recommandé que les badges soient visuellement les plus neutres possibles. Ils ne doivent notamment pas indiquer:
+* d'informations sur l'entreprise (nom, adresse) &lt;abbr title="Si des coordonnées sont indiquées sur le dos du badge pour faciliter sa restitution en cas de perte, elles ne doivent pas mentionner explicitement le nom de l&amp;#x27;entité. Mieux vaut privilégier dans ce cas l&amp;#x27;utilisation d&amp;#x27;une boîte postale."&gt;&lt;sup&gt;24&lt;/sup&gt;&lt;/abbr&gt;;
+* d'informations sur le porteur (nom, prénom, poste), en dehors de sa photo;
+* les accès autorisés. Un numéro de traçabilité peut être indiqué sur le badge à des fins administratives, mais ce numéro doit être différent du numéro d'identification. La photographie est tolérée car elle permet de vérifier rapidement que le badge appartient bien au porteur.</t>
   </si>
 </sst>
 </file>
@@ -2588,7 +2588,7 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="302.39999999999998" x14ac:dyDescent="0.3">
@@ -2674,7 +2674,7 @@
         <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="273.60000000000002" x14ac:dyDescent="0.3">
@@ -2745,7 +2745,7 @@
         <v>30</v>
       </c>
       <c r="E2" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2756,7 +2756,7 @@
         <v>31</v>
       </c>
       <c r="E3" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -2773,7 +2773,7 @@
         <v>35</v>
       </c>
       <c r="E4" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>477</v>
@@ -2793,7 +2793,7 @@
         <v>33</v>
       </c>
       <c r="E5" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
@@ -2804,7 +2804,7 @@
         <v>37</v>
       </c>
       <c r="E6" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
@@ -2821,7 +2821,7 @@
         <v>39</v>
       </c>
       <c r="E7" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>40</v>
@@ -2838,7 +2838,7 @@
         <v>41</v>
       </c>
       <c r="E8" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -2855,7 +2855,7 @@
         <v>43</v>
       </c>
       <c r="E9" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>44</v>
@@ -2872,7 +2872,7 @@
         <v>45</v>
       </c>
       <c r="E10" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -2889,7 +2889,7 @@
         <v>47</v>
       </c>
       <c r="E11" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>48</v>
@@ -2912,7 +2912,7 @@
         <v>50</v>
       </c>
       <c r="E12" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>51</v>
@@ -2929,7 +2929,7 @@
         <v>52</v>
       </c>
       <c r="E13" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -2946,7 +2946,7 @@
         <v>54</v>
       </c>
       <c r="E14" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>55</v>
@@ -2963,7 +2963,7 @@
         <v>56</v>
       </c>
       <c r="E15" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
@@ -2980,7 +2980,7 @@
         <v>58</v>
       </c>
       <c r="E16" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>59</v>
@@ -2997,7 +2997,7 @@
         <v>60</v>
       </c>
       <c r="E17" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -3014,7 +3014,7 @@
         <v>62</v>
       </c>
       <c r="E18" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>63</v>
@@ -3031,7 +3031,7 @@
         <v>64</v>
       </c>
       <c r="E19" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -3048,7 +3048,7 @@
         <v>66</v>
       </c>
       <c r="E20" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>67</v>
@@ -3065,7 +3065,7 @@
         <v>68</v>
       </c>
       <c r="E21" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
@@ -3076,7 +3076,7 @@
         <v>69</v>
       </c>
       <c r="E22" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -3093,7 +3093,7 @@
         <v>71</v>
       </c>
       <c r="E23" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="F23" s="1" t="s">
         <v>72</v>
@@ -3116,7 +3116,7 @@
         <v>74</v>
       </c>
       <c r="E24" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>75</v>
@@ -3139,7 +3139,7 @@
         <v>78</v>
       </c>
       <c r="E25" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="F25" s="1" t="s">
         <v>79</v>
@@ -3156,7 +3156,7 @@
         <v>80</v>
       </c>
       <c r="E26" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
@@ -3167,7 +3167,7 @@
         <v>81</v>
       </c>
       <c r="E27" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -3184,7 +3184,7 @@
         <v>83</v>
       </c>
       <c r="E28" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>84</v>
@@ -3201,7 +3201,7 @@
         <v>85</v>
       </c>
       <c r="E29" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -3218,7 +3218,7 @@
         <v>87</v>
       </c>
       <c r="E30" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="F30" s="1" t="s">
         <v>88</v>
@@ -3241,7 +3241,7 @@
         <v>90</v>
       </c>
       <c r="E31" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="F31" s="1" t="s">
         <v>91</v>
@@ -3258,7 +3258,7 @@
         <v>92</v>
       </c>
       <c r="E32" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -3275,7 +3275,7 @@
         <v>94</v>
       </c>
       <c r="E33" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="F33" s="1" t="s">
         <v>95</v>
@@ -3298,7 +3298,7 @@
         <v>97</v>
       </c>
       <c r="E34" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="F34" s="1" t="s">
         <v>98</v>
@@ -3315,7 +3315,7 @@
         <v>99</v>
       </c>
       <c r="E35" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.3">
@@ -3326,7 +3326,7 @@
         <v>100</v>
       </c>
       <c r="E36" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -3343,7 +3343,7 @@
         <v>102</v>
       </c>
       <c r="E37" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="F37" s="1" t="s">
         <v>103</v>
@@ -3360,7 +3360,7 @@
         <v>104</v>
       </c>
       <c r="E38" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -3377,7 +3377,7 @@
         <v>106</v>
       </c>
       <c r="E39" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="F39" s="1" t="s">
         <v>107</v>
@@ -3400,7 +3400,7 @@
         <v>109</v>
       </c>
       <c r="E40" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="F40" s="1" t="s">
         <v>110</v>
@@ -3423,7 +3423,7 @@
         <v>112</v>
       </c>
       <c r="E41" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="F41" s="1" t="s">
         <v>113</v>
@@ -3446,7 +3446,7 @@
         <v>115</v>
       </c>
       <c r="E42" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="F42" s="1" t="s">
         <v>116</v>
@@ -3463,7 +3463,7 @@
         <v>117</v>
       </c>
       <c r="E43" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
     </row>
     <row r="44" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -3480,7 +3480,7 @@
         <v>119</v>
       </c>
       <c r="E44" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="F44" s="1" t="s">
         <v>120</v>
@@ -3497,7 +3497,7 @@
         <v>121</v>
       </c>
       <c r="E45" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.3">
@@ -3514,7 +3514,7 @@
         <v>123</v>
       </c>
       <c r="E46" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="F46" s="1" t="s">
         <v>124</v>
@@ -3537,7 +3537,7 @@
         <v>126</v>
       </c>
       <c r="E47" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="F47" s="1" t="s">
         <v>127</v>
@@ -3557,7 +3557,7 @@
         <v>128</v>
       </c>
       <c r="E48" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
     </row>
     <row r="49" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -3574,7 +3574,7 @@
         <v>130</v>
       </c>
       <c r="E49" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="F49" s="1" t="s">
         <v>131</v>
@@ -3597,7 +3597,7 @@
         <v>133</v>
       </c>
       <c r="E50" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="F50" s="1" t="s">
         <v>134</v>
@@ -3614,7 +3614,7 @@
         <v>135</v>
       </c>
       <c r="E51" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.3">
@@ -3625,7 +3625,7 @@
         <v>136</v>
       </c>
       <c r="E52" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
     </row>
     <row r="53" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -3642,7 +3642,7 @@
         <v>138</v>
       </c>
       <c r="E53" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="F53" s="1" t="s">
         <v>139</v>
@@ -3659,7 +3659,7 @@
         <v>140</v>
       </c>
       <c r="E54" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
     </row>
     <row r="55" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
@@ -3676,7 +3676,7 @@
         <v>142</v>
       </c>
       <c r="E55" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="F55" s="1" t="s">
         <v>479</v>
@@ -3693,7 +3693,7 @@
         <v>143</v>
       </c>
       <c r="E56" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
     </row>
     <row r="57" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -3710,7 +3710,7 @@
         <v>145</v>
       </c>
       <c r="E57" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="F57" s="1" t="s">
         <v>146</v>
@@ -3727,7 +3727,7 @@
         <v>147</v>
       </c>
       <c r="E58" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.3">
@@ -3744,7 +3744,7 @@
         <v>149</v>
       </c>
       <c r="E59" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="F59" s="1" t="s">
         <v>150</v>
@@ -3767,7 +3767,7 @@
         <v>152</v>
       </c>
       <c r="E60" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="F60" s="1" t="s">
         <v>153</v>
@@ -3787,7 +3787,7 @@
         <v>154</v>
       </c>
       <c r="E61" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.3">
@@ -3798,7 +3798,7 @@
         <v>155</v>
       </c>
       <c r="E62" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.3">
@@ -3815,7 +3815,7 @@
         <v>157</v>
       </c>
       <c r="E63" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="F63" s="1" t="s">
         <v>158</v>
@@ -3838,7 +3838,7 @@
         <v>160</v>
       </c>
       <c r="E64" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="F64" s="1" t="s">
         <v>161</v>
@@ -3861,7 +3861,7 @@
         <v>163</v>
       </c>
       <c r="E65" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="F65" s="1" t="s">
         <v>164</v>
@@ -3881,7 +3881,7 @@
         <v>165</v>
       </c>
       <c r="E66" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
     </row>
     <row r="67" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -3898,7 +3898,7 @@
         <v>167</v>
       </c>
       <c r="E67" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="F67" s="1" t="s">
         <v>168</v>
@@ -3921,7 +3921,7 @@
         <v>170</v>
       </c>
       <c r="E68" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="F68" s="1" t="s">
         <v>171</v>
@@ -3938,7 +3938,7 @@
         <v>172</v>
       </c>
       <c r="E69" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.3">
@@ -3949,7 +3949,7 @@
         <v>173</v>
       </c>
       <c r="E70" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
     <row r="71" spans="1:8" ht="158.4" x14ac:dyDescent="0.3">
@@ -3966,7 +3966,7 @@
         <v>175</v>
       </c>
       <c r="E71" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="F71" s="1" t="s">
         <v>480</v>
@@ -3983,7 +3983,7 @@
         <v>176</v>
       </c>
       <c r="E72" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.3">
@@ -3994,7 +3994,7 @@
         <v>177</v>
       </c>
       <c r="E73" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
     </row>
     <row r="74" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
@@ -4011,7 +4011,7 @@
         <v>179</v>
       </c>
       <c r="E74" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="F74" s="1" t="s">
         <v>180</v>
@@ -4037,7 +4037,7 @@
         <v>182</v>
       </c>
       <c r="E75" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="F75" s="1" t="s">
         <v>183</v>
@@ -4046,7 +4046,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="76" spans="1:8" ht="172.8" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>32</v>
       </c>
@@ -4060,10 +4060,10 @@
         <v>185</v>
       </c>
       <c r="E76" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="F76" s="1" t="s">
-        <v>481</v>
+        <v>696</v>
       </c>
       <c r="H76" t="s">
         <v>36</v>
@@ -4083,7 +4083,7 @@
         <v>187</v>
       </c>
       <c r="E77" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="F77" s="1" t="s">
         <v>188</v>
@@ -4106,7 +4106,7 @@
         <v>190</v>
       </c>
       <c r="E78" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="F78" s="1" t="s">
         <v>191</v>
@@ -4123,7 +4123,7 @@
         <v>192</v>
       </c>
       <c r="E79" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
     </row>
     <row r="80" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -4140,7 +4140,7 @@
         <v>194</v>
       </c>
       <c r="E80" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="F80" s="1" t="s">
         <v>195</v>
@@ -4157,7 +4157,7 @@
         <v>196</v>
       </c>
       <c r="E81" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
     </row>
     <row r="82" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -4174,7 +4174,7 @@
         <v>198</v>
       </c>
       <c r="E82" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="F82" s="1" t="s">
         <v>199</v>
@@ -4197,7 +4197,7 @@
         <v>201</v>
       </c>
       <c r="E83" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="F83" s="1" t="s">
         <v>202</v>
@@ -4214,7 +4214,7 @@
         <v>203</v>
       </c>
       <c r="E84" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
     </row>
     <row r="85" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -4231,7 +4231,7 @@
         <v>205</v>
       </c>
       <c r="E85" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="F85" s="1" t="s">
         <v>206</v>
@@ -4254,7 +4254,7 @@
         <v>208</v>
       </c>
       <c r="E86" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="F86" s="1" t="s">
         <v>209</v>
@@ -4277,7 +4277,7 @@
         <v>211</v>
       </c>
       <c r="E87" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="F87" s="1" t="s">
         <v>212</v>
@@ -4294,7 +4294,7 @@
         <v>213</v>
       </c>
       <c r="E88" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
     </row>
     <row r="89" spans="1:8" ht="72" x14ac:dyDescent="0.3">
@@ -4311,7 +4311,7 @@
         <v>215</v>
       </c>
       <c r="E89" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="F89" s="1" t="s">
         <v>216</v>
@@ -4328,7 +4328,7 @@
         <v>217</v>
       </c>
       <c r="E90" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="91" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -4345,7 +4345,7 @@
         <v>219</v>
       </c>
       <c r="E91" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="F91" s="1" t="s">
         <v>220</v>
@@ -4362,7 +4362,7 @@
         <v>221</v>
       </c>
       <c r="E92" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="93" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -4379,7 +4379,7 @@
         <v>223</v>
       </c>
       <c r="E93" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="F93" s="1" t="s">
         <v>224</v>
@@ -4402,7 +4402,7 @@
         <v>226</v>
       </c>
       <c r="E94" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="F94" s="1" t="s">
         <v>227</v>
@@ -4419,7 +4419,7 @@
         <v>228</v>
       </c>
       <c r="E95" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
     <row r="96" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -4436,7 +4436,7 @@
         <v>230</v>
       </c>
       <c r="E96" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="F96" s="1" t="s">
         <v>231</v>
@@ -4459,7 +4459,7 @@
         <v>233</v>
       </c>
       <c r="E97" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="F97" s="1" t="s">
         <v>234</v>
@@ -4482,7 +4482,7 @@
         <v>237</v>
       </c>
       <c r="E98" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="F98" s="1" t="s">
         <v>238</v>
@@ -4508,7 +4508,7 @@
         <v>240</v>
       </c>
       <c r="E99" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="F99" s="1" t="s">
         <v>241</v>
@@ -4531,7 +4531,7 @@
         <v>243</v>
       </c>
       <c r="E100" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="F100" s="1" t="s">
         <v>244</v>
@@ -4554,7 +4554,7 @@
         <v>246</v>
       </c>
       <c r="E101" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="F101" s="1" t="s">
         <v>247</v>
@@ -4571,7 +4571,7 @@
         <v>248</v>
       </c>
       <c r="E102" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
     </row>
     <row r="103" spans="1:8" x14ac:dyDescent="0.3">
@@ -4582,7 +4582,7 @@
         <v>249</v>
       </c>
       <c r="E103" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="104" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -4599,7 +4599,7 @@
         <v>251</v>
       </c>
       <c r="E104" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="F104" s="1" t="s">
         <v>252</v>
@@ -4622,7 +4622,7 @@
         <v>254</v>
       </c>
       <c r="E105" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="F105" s="1" t="s">
         <v>255</v>
@@ -4645,7 +4645,7 @@
         <v>257</v>
       </c>
       <c r="E106" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="F106" s="1" t="s">
         <v>258</v>
@@ -4668,7 +4668,7 @@
         <v>260</v>
       </c>
       <c r="E107" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="F107" s="1" t="s">
         <v>261</v>
@@ -4691,7 +4691,7 @@
         <v>263</v>
       </c>
       <c r="E108" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="F108" s="1" t="s">
         <v>264</v>
@@ -4714,10 +4714,10 @@
         <v>266</v>
       </c>
       <c r="E109" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="F109" s="1" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="H109" t="s">
         <v>36</v>
@@ -4731,7 +4731,7 @@
         <v>267</v>
       </c>
       <c r="E110" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
     </row>
     <row r="111" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -4748,7 +4748,7 @@
         <v>269</v>
       </c>
       <c r="E111" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="F111" s="1" t="s">
         <v>270</v>
@@ -4771,7 +4771,7 @@
         <v>272</v>
       </c>
       <c r="E112" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="F112" s="1" t="s">
         <v>273</v>
@@ -4794,7 +4794,7 @@
         <v>275</v>
       </c>
       <c r="E113" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="F113" s="1" t="s">
         <v>276</v>
@@ -4820,7 +4820,7 @@
         <v>278</v>
       </c>
       <c r="E114" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="F114" s="1" t="s">
         <v>279</v>
@@ -4843,7 +4843,7 @@
         <v>281</v>
       </c>
       <c r="E115" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="F115" s="1" t="s">
         <v>282</v>
@@ -4866,7 +4866,7 @@
         <v>284</v>
       </c>
       <c r="E116" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="F116" s="1" t="s">
         <v>285</v>
@@ -4889,7 +4889,7 @@
         <v>287</v>
       </c>
       <c r="E117" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="F117" s="1" t="s">
         <v>288</v>
@@ -4906,7 +4906,7 @@
         <v>289</v>
       </c>
       <c r="E118" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
     </row>
     <row r="119" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -4923,7 +4923,7 @@
         <v>291</v>
       </c>
       <c r="E119" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="F119" s="1" t="s">
         <v>292</v>
@@ -4940,7 +4940,7 @@
         <v>293</v>
       </c>
       <c r="E120" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
     </row>
     <row r="121" spans="1:8" x14ac:dyDescent="0.3">
@@ -4951,7 +4951,7 @@
         <v>294</v>
       </c>
       <c r="E121" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
     </row>
     <row r="122" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -4968,7 +4968,7 @@
         <v>296</v>
       </c>
       <c r="E122" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="F122" s="1" t="s">
         <v>297</v>
@@ -4985,7 +4985,7 @@
         <v>298</v>
       </c>
       <c r="E123" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
     </row>
     <row r="124" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -5002,7 +5002,7 @@
         <v>300</v>
       </c>
       <c r="E124" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="F124" s="1" t="s">
         <v>301</v>
@@ -5019,7 +5019,7 @@
         <v>302</v>
       </c>
       <c r="E125" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
     </row>
     <row r="126" spans="1:8" ht="72" x14ac:dyDescent="0.3">
@@ -5036,7 +5036,7 @@
         <v>304</v>
       </c>
       <c r="E126" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="F126" s="1" t="s">
         <v>305</v>
@@ -5059,7 +5059,7 @@
         <v>307</v>
       </c>
       <c r="E127" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="F127" s="1" t="s">
         <v>308</v>
@@ -5076,7 +5076,7 @@
         <v>309</v>
       </c>
       <c r="E128" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
     </row>
     <row r="129" spans="1:8" x14ac:dyDescent="0.3">
@@ -5087,7 +5087,7 @@
         <v>310</v>
       </c>
       <c r="E129" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
     </row>
     <row r="130" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -5104,7 +5104,7 @@
         <v>312</v>
       </c>
       <c r="E130" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="F130" s="1" t="s">
         <v>313</v>
@@ -5121,7 +5121,7 @@
         <v>314</v>
       </c>
       <c r="E131" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="132" spans="1:8" x14ac:dyDescent="0.3">
@@ -5138,7 +5138,7 @@
         <v>316</v>
       </c>
       <c r="E132" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="F132" s="1" t="s">
         <v>317</v>
@@ -5161,7 +5161,7 @@
         <v>319</v>
       </c>
       <c r="E133" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="F133" s="1" t="s">
         <v>320</v>
@@ -5178,7 +5178,7 @@
         <v>321</v>
       </c>
       <c r="E134" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
     </row>
     <row r="135" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -5195,7 +5195,7 @@
         <v>323</v>
       </c>
       <c r="E135" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="F135" s="1" t="s">
         <v>324</v>
@@ -5218,7 +5218,7 @@
         <v>326</v>
       </c>
       <c r="E136" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="F136" s="1" t="s">
         <v>327</v>
@@ -5235,7 +5235,7 @@
         <v>328</v>
       </c>
       <c r="E137" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
     </row>
     <row r="138" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -5252,7 +5252,7 @@
         <v>330</v>
       </c>
       <c r="E138" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="F138" s="1" t="s">
         <v>331</v>
@@ -5269,7 +5269,7 @@
         <v>332</v>
       </c>
       <c r="E139" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
     </row>
     <row r="140" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -5286,7 +5286,7 @@
         <v>334</v>
       </c>
       <c r="E140" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="F140" s="1" t="s">
         <v>335</v>
@@ -5309,7 +5309,7 @@
         <v>337</v>
       </c>
       <c r="E141" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="F141" s="1" t="s">
         <v>338</v>
@@ -5332,7 +5332,7 @@
         <v>340</v>
       </c>
       <c r="E142" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F142" s="1" t="s">
         <v>341</v>
@@ -5349,7 +5349,7 @@
         <v>342</v>
       </c>
       <c r="E143" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
     </row>
     <row r="144" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -5366,7 +5366,7 @@
         <v>344</v>
       </c>
       <c r="E144" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="F144" s="1" t="s">
         <v>345</v>
@@ -5383,7 +5383,7 @@
         <v>346</v>
       </c>
       <c r="E145" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
     </row>
     <row r="146" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
@@ -5400,7 +5400,7 @@
         <v>348</v>
       </c>
       <c r="E146" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="F146" s="1" t="s">
         <v>349</v>
@@ -5417,7 +5417,7 @@
         <v>350</v>
       </c>
       <c r="E147" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
     </row>
     <row r="148" spans="1:8" x14ac:dyDescent="0.3">
@@ -5428,7 +5428,7 @@
         <v>351</v>
       </c>
       <c r="E148" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
     </row>
     <row r="149" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -5445,7 +5445,7 @@
         <v>353</v>
       </c>
       <c r="E149" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="F149" s="1" t="s">
         <v>354</v>
@@ -5462,7 +5462,7 @@
         <v>355</v>
       </c>
       <c r="E150" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
     </row>
     <row r="151" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -5479,7 +5479,7 @@
         <v>357</v>
       </c>
       <c r="E151" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="F151" s="1" t="s">
         <v>358</v>
@@ -5496,7 +5496,7 @@
         <v>359</v>
       </c>
       <c r="E152" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
     </row>
     <row r="153" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -5513,7 +5513,7 @@
         <v>361</v>
       </c>
       <c r="E153" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="F153" s="1" t="s">
         <v>362</v>
@@ -5536,7 +5536,7 @@
         <v>364</v>
       </c>
       <c r="E154" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="F154" s="1" t="s">
         <v>365</v>
@@ -5553,7 +5553,7 @@
         <v>366</v>
       </c>
       <c r="E155" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
     </row>
     <row r="156" spans="1:8" x14ac:dyDescent="0.3">
@@ -5564,7 +5564,7 @@
         <v>367</v>
       </c>
       <c r="E156" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
     </row>
     <row r="157" spans="1:8" x14ac:dyDescent="0.3">
@@ -5575,7 +5575,7 @@
         <v>368</v>
       </c>
       <c r="E157" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
     </row>
     <row r="158" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -5592,7 +5592,7 @@
         <v>370</v>
       </c>
       <c r="E158" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="F158" s="1" t="s">
         <v>371</v>
@@ -5615,7 +5615,7 @@
         <v>373</v>
       </c>
       <c r="E159" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="F159" s="1" t="s">
         <v>374</v>
@@ -5632,7 +5632,7 @@
         <v>375</v>
       </c>
       <c r="E160" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
     </row>
     <row r="161" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -5649,7 +5649,7 @@
         <v>377</v>
       </c>
       <c r="E161" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="F161" s="1" t="s">
         <v>378</v>
@@ -5666,7 +5666,7 @@
         <v>379</v>
       </c>
       <c r="E162" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
     </row>
     <row r="163" spans="1:8" x14ac:dyDescent="0.3">
@@ -5677,7 +5677,7 @@
         <v>380</v>
       </c>
       <c r="E163" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
     </row>
     <row r="164" spans="1:8" ht="72" x14ac:dyDescent="0.3">
@@ -5694,10 +5694,10 @@
         <v>382</v>
       </c>
       <c r="E164" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="F164" s="1" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="H164" t="s">
         <v>36</v>
@@ -5711,7 +5711,7 @@
         <v>383</v>
       </c>
       <c r="E165" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
     </row>
     <row r="166" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -5728,7 +5728,7 @@
         <v>385</v>
       </c>
       <c r="E166" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="F166" s="1" t="s">
         <v>386</v>
@@ -5745,7 +5745,7 @@
         <v>387</v>
       </c>
       <c r="E167" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
     </row>
     <row r="168" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -5762,7 +5762,7 @@
         <v>389</v>
       </c>
       <c r="E168" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="F168" s="1" t="s">
         <v>390</v>
@@ -5779,7 +5779,7 @@
         <v>391</v>
       </c>
       <c r="E169" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
     </row>
     <row r="170" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -5796,7 +5796,7 @@
         <v>393</v>
       </c>
       <c r="E170" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="F170" s="1" t="s">
         <v>394</v>
@@ -5813,7 +5813,7 @@
         <v>395</v>
       </c>
       <c r="E171" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
     </row>
     <row r="172" spans="1:8" x14ac:dyDescent="0.3">
@@ -5824,7 +5824,7 @@
         <v>396</v>
       </c>
       <c r="E172" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
     </row>
     <row r="173" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -5841,7 +5841,7 @@
         <v>398</v>
       </c>
       <c r="E173" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="F173" s="1" t="s">
         <v>399</v>
@@ -5858,7 +5858,7 @@
         <v>400</v>
       </c>
       <c r="E174" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
     </row>
     <row r="175" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
@@ -5875,10 +5875,10 @@
         <v>402</v>
       </c>
       <c r="E175" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="F175" s="1" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="H175" t="s">
         <v>36</v>
@@ -5892,7 +5892,7 @@
         <v>403</v>
       </c>
       <c r="E176" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
     </row>
     <row r="177" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -5909,7 +5909,7 @@
         <v>405</v>
       </c>
       <c r="E177" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="F177" s="1" t="s">
         <v>406</v>
@@ -5932,7 +5932,7 @@
         <v>408</v>
       </c>
       <c r="E178" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="F178" s="1" t="s">
         <v>409</v>
@@ -5955,7 +5955,7 @@
         <v>411</v>
       </c>
       <c r="E179" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="F179" s="1" t="s">
         <v>412</v>
@@ -5972,7 +5972,7 @@
         <v>413</v>
       </c>
       <c r="E180" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
     </row>
     <row r="181" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -5989,7 +5989,7 @@
         <v>415</v>
       </c>
       <c r="E181" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="F181" s="1" t="s">
         <v>416</v>
@@ -6006,7 +6006,7 @@
         <v>417</v>
       </c>
       <c r="E182" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
     </row>
     <row r="183" spans="1:8" x14ac:dyDescent="0.3">
@@ -6017,7 +6017,7 @@
         <v>418</v>
       </c>
       <c r="E183" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
     </row>
     <row r="184" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -6034,7 +6034,7 @@
         <v>420</v>
       </c>
       <c r="E184" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="F184" s="1" t="s">
         <v>421</v>
@@ -6057,7 +6057,7 @@
         <v>423</v>
       </c>
       <c r="E185" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="F185" s="1" t="s">
         <v>424</v>
@@ -6080,7 +6080,7 @@
         <v>426</v>
       </c>
       <c r="E186" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="F186" s="1" t="s">
         <v>427</v>
@@ -6097,7 +6097,7 @@
         <v>428</v>
       </c>
       <c r="E187" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
     </row>
     <row r="188" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -6114,7 +6114,7 @@
         <v>430</v>
       </c>
       <c r="E188" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="F188" s="1" t="s">
         <v>431</v>
@@ -6131,7 +6131,7 @@
         <v>432</v>
       </c>
       <c r="E189" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
     </row>
     <row r="190" spans="1:8" x14ac:dyDescent="0.3">
@@ -6142,7 +6142,7 @@
         <v>433</v>
       </c>
       <c r="E190" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
     </row>
     <row r="191" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -6159,7 +6159,7 @@
         <v>435</v>
       </c>
       <c r="E191" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="F191" s="1" t="s">
         <v>436</v>
@@ -6176,7 +6176,7 @@
         <v>437</v>
       </c>
       <c r="E192" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
     </row>
     <row r="193" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -6193,10 +6193,10 @@
         <v>439</v>
       </c>
       <c r="E193" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="F193" s="1" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="H193" t="s">
         <v>36</v>
@@ -6210,7 +6210,7 @@
         <v>440</v>
       </c>
       <c r="E194" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
     </row>
     <row r="195" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -6227,7 +6227,7 @@
         <v>442</v>
       </c>
       <c r="E195" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="F195" s="1" t="s">
         <v>443</v>
@@ -6244,7 +6244,7 @@
         <v>444</v>
       </c>
       <c r="E196" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
     </row>
     <row r="197" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
@@ -6261,7 +6261,7 @@
         <v>446</v>
       </c>
       <c r="E197" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="F197" s="1" t="s">
         <v>447</v>
@@ -6278,7 +6278,7 @@
         <v>448</v>
       </c>
       <c r="E198" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
     </row>
     <row r="199" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -6295,7 +6295,7 @@
         <v>450</v>
       </c>
       <c r="E199" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="F199" s="1" t="s">
         <v>451</v>
@@ -6312,7 +6312,7 @@
         <v>452</v>
       </c>
       <c r="E200" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
     </row>
     <row r="201" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -6329,7 +6329,7 @@
         <v>454</v>
       </c>
       <c r="E201" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="F201" s="1" t="s">
         <v>455</v>
@@ -6346,7 +6346,7 @@
         <v>456</v>
       </c>
       <c r="E202" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
     </row>
     <row r="203" spans="1:8" x14ac:dyDescent="0.3">
@@ -6357,7 +6357,7 @@
         <v>457</v>
       </c>
       <c r="E203" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
     </row>
     <row r="204" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -6374,7 +6374,7 @@
         <v>459</v>
       </c>
       <c r="E204" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="F204" s="1" t="s">
         <v>460</v>
@@ -6391,7 +6391,7 @@
         <v>461</v>
       </c>
       <c r="E205" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
     </row>
     <row r="206" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -6408,7 +6408,7 @@
         <v>463</v>
       </c>
       <c r="E206" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="F206" s="1" t="s">
         <v>464</v>
@@ -6425,7 +6425,7 @@
         <v>465</v>
       </c>
       <c r="E207" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
     </row>
     <row r="208" spans="1:8" x14ac:dyDescent="0.3">
@@ -6442,7 +6442,7 @@
         <v>467</v>
       </c>
       <c r="E208" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="F208" s="1" t="s">
         <v>468</v>
@@ -6513,7 +6513,7 @@
         <v>36</v>
       </c>
       <c r="B2" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="C2" t="s">
         <v>469</v>
@@ -6524,7 +6524,7 @@
         <v>76</v>
       </c>
       <c r="B3" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="C3" t="s">
         <v>470</v>
@@ -6535,7 +6535,7 @@
         <v>235</v>
       </c>
       <c r="B4" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>471</v>

</xml_diff>